<commit_message>
Weekly League One data update: 2026-09-26
</commit_message>
<xml_diff>
--- a/data/league-one_xg_report.xlsx
+++ b/data/league-one_xg_report.xlsx
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1.42</v>
+        <v>1.38</v>
       </c>
       <c r="C2" s="9" t="n">
         <v>0.34</v>
@@ -1232,7 +1232,7 @@
         <v>2.47</v>
       </c>
       <c r="F2" s="9" t="n">
-        <v>1.37</v>
+        <v>1.2</v>
       </c>
       <c r="G2" s="6" t="n"/>
     </row>
@@ -1260,45 +1260,45 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Peterborough United</t>
+          <t>Doncaster Rovers</t>
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>0.39</v>
+        <v>0.37</v>
       </c>
       <c r="C4" s="9" t="n">
-        <v>0.31</v>
+        <v>0.9</v>
       </c>
       <c r="D4" s="9" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="F4" s="9" t="n">
-        <v>0.06</v>
-      </c>
+        <v>0.2</v>
+      </c>
+      <c r="F4" s="6" t="n"/>
       <c r="G4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Doncaster Rovers</t>
+          <t>Peterborough United</t>
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>0.37</v>
+        <v>0.35</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>0.9</v>
+        <v>0.31</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F5" s="6" t="n"/>
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>-0.11</v>
+      </c>
       <c r="G5" s="6" t="n"/>
     </row>
     <row r="6">
@@ -1352,7 +1352,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>0.21</v>
+        <v>0.23</v>
       </c>
       <c r="C8" s="9" t="n">
         <v>0.8100000000000001</v>
@@ -1364,7 +1364,7 @@
         <v>-1.76</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>-0.2</v>
+        <v>-0.12</v>
       </c>
       <c r="G8" s="6" t="n"/>
     </row>
@@ -1459,7 +1459,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>-0.19</v>
+        <v>-0.2</v>
       </c>
       <c r="C13" s="9" t="n">
         <v>0.18</v>
@@ -1471,7 +1471,7 @@
         <v>1.01</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>-0.99</v>
+        <v>-1.04</v>
       </c>
       <c r="G13" s="6" t="n"/>
     </row>
@@ -1882,7 +1882,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>0.6</v>
+        <v>0.58</v>
       </c>
       <c r="C5" s="9" t="n">
         <v>1.26</v>
@@ -1894,7 +1894,7 @@
         <v>1.3</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>0.2</v>
+        <v>0.12</v>
       </c>
       <c r="G5" s="6" t="n"/>
     </row>
@@ -1926,7 +1926,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>0.5</v>
+        <v>0.54</v>
       </c>
       <c r="C7" s="9" t="n">
         <v>-0.01</v>
@@ -1938,7 +1938,7 @@
         <v>1.6</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>-0.06</v>
+        <v>0.11</v>
       </c>
       <c r="G7" s="6" t="n"/>
     </row>
@@ -2169,67 +2169,67 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Bromley</t>
+          <t>Notts County</t>
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>-0.18</v>
+        <v>-0.14</v>
       </c>
       <c r="C18" s="9" t="n">
-        <v>0.48</v>
+        <v>-0.16</v>
       </c>
       <c r="D18" s="9" t="n">
-        <v>-2</v>
+        <v>-0</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="F18" s="6" t="n"/>
+        <v>0.78</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>-1.2</v>
+      </c>
       <c r="G18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Leicester City</t>
+          <t>Bromley</t>
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>-0.19</v>
+        <v>-0.18</v>
       </c>
       <c r="C19" s="9" t="n">
-        <v>-1.91</v>
+        <v>0.48</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>0.82</v>
+        <v>-2</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>-0.44</v>
-      </c>
-      <c r="F19" s="9" t="n">
-        <v>0.76</v>
-      </c>
+        <v>0.98</v>
+      </c>
+      <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Notts County</t>
+          <t>Leicester City</t>
         </is>
       </c>
       <c r="B20" s="13" t="n">
         <v>-0.19</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>-0.16</v>
+        <v>-1.91</v>
       </c>
       <c r="D20" s="9" t="n">
-        <v>-0</v>
+        <v>0.82</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>0.78</v>
+        <v>-0.44</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>-1.37</v>
+        <v>0.76</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -2240,7 +2240,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>-0.22</v>
+        <v>-0.21</v>
       </c>
       <c r="C21" s="9" t="n">
         <v>-0.31</v>
@@ -2252,7 +2252,7 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>0.99</v>
+        <v>1.04</v>
       </c>
       <c r="G21" s="6" t="n"/>
     </row>
@@ -2530,85 +2530,85 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Reading</t>
+          <t>Sheffield Wednesday</t>
         </is>
       </c>
       <c r="B4" s="13">
-        <f>'Reading'!$E$23</f>
+        <f>'Sheffield Wednesday'!$E$24</f>
         <v/>
       </c>
       <c r="C4" s="9">
-        <f>'Reading'!$S$2</f>
+        <f>'Sheffield Wednesday'!$S$2</f>
         <v/>
       </c>
       <c r="D4" s="9">
-        <f>'Reading'!$S$3</f>
+        <f>'Sheffield Wednesday'!$S$3</f>
         <v/>
       </c>
       <c r="E4" s="9">
-        <f>'Reading'!$S$4</f>
+        <f>'Sheffield Wednesday'!$S$4</f>
         <v/>
       </c>
       <c r="F4" s="9">
-        <f>'Reading'!$S$5</f>
+        <f>'Sheffield Wednesday'!$S$5</f>
         <v/>
       </c>
       <c r="G4" s="9">
-        <f>'Reading'!$S$6</f>
+        <f>'Sheffield Wednesday'!$S$6</f>
         <v/>
       </c>
       <c r="H4" s="9">
-        <f>'Reading'!$S$7</f>
-        <v/>
-      </c>
-      <c r="I4" s="6" t="n"/>
+        <f>'Sheffield Wednesday'!$S$7</f>
+        <v/>
+      </c>
+      <c r="I4" s="9">
+        <f>'Sheffield Wednesday'!$S$8</f>
+        <v/>
+      </c>
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="13">
-        <f>'Reading'!$E$24</f>
+        <f>'Sheffield Wednesday'!$E$25</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Sheffield Wednesday</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B5" s="13">
-        <f>'Sheffield Wednesday'!$E$24</f>
+        <f>'Reading'!$E$23</f>
         <v/>
       </c>
       <c r="C5" s="9">
-        <f>'Sheffield Wednesday'!$S$2</f>
+        <f>'Reading'!$S$2</f>
         <v/>
       </c>
       <c r="D5" s="9">
-        <f>'Sheffield Wednesday'!$S$3</f>
+        <f>'Reading'!$S$3</f>
         <v/>
       </c>
       <c r="E5" s="9">
-        <f>'Sheffield Wednesday'!$S$4</f>
+        <f>'Reading'!$S$4</f>
         <v/>
       </c>
       <c r="F5" s="9">
-        <f>'Sheffield Wednesday'!$S$5</f>
+        <f>'Reading'!$S$5</f>
         <v/>
       </c>
       <c r="G5" s="9">
-        <f>'Sheffield Wednesday'!$S$6</f>
+        <f>'Reading'!$S$6</f>
         <v/>
       </c>
       <c r="H5" s="9">
-        <f>'Sheffield Wednesday'!$S$7</f>
-        <v/>
-      </c>
-      <c r="I5" s="9">
-        <f>'Sheffield Wednesday'!$S$8</f>
-        <v/>
-      </c>
+        <f>'Reading'!$S$7</f>
+        <v/>
+      </c>
+      <c r="I5" s="6" t="n"/>
       <c r="J5" s="6" t="n"/>
       <c r="K5" s="13">
-        <f>'Sheffield Wednesday'!$E$25</f>
+        <f>'Reading'!$E$24</f>
         <v/>
       </c>
     </row>
@@ -2967,220 +2967,220 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Leyton Orient</t>
+          <t>Doncaster Rovers</t>
         </is>
       </c>
       <c r="B14" s="13">
-        <f>'Leyton Orient'!$E$24</f>
+        <f>'Doncaster Rovers'!$E$24</f>
         <v/>
       </c>
       <c r="C14" s="9">
-        <f>'Leyton Orient'!$S$2</f>
+        <f>'Doncaster Rovers'!$S$2</f>
         <v/>
       </c>
       <c r="D14" s="9">
-        <f>'Leyton Orient'!$S$3</f>
+        <f>'Doncaster Rovers'!$S$3</f>
         <v/>
       </c>
       <c r="E14" s="9">
-        <f>'Leyton Orient'!$S$4</f>
+        <f>'Doncaster Rovers'!$S$4</f>
         <v/>
       </c>
       <c r="F14" s="9">
-        <f>'Leyton Orient'!$S$5</f>
+        <f>'Doncaster Rovers'!$S$5</f>
         <v/>
       </c>
       <c r="G14" s="9">
-        <f>'Leyton Orient'!$S$6</f>
+        <f>'Doncaster Rovers'!$S$6</f>
         <v/>
       </c>
       <c r="H14" s="9">
-        <f>'Leyton Orient'!$S$7</f>
+        <f>'Doncaster Rovers'!$S$7</f>
         <v/>
       </c>
       <c r="I14" s="9">
-        <f>'Leyton Orient'!$S$8</f>
+        <f>'Doncaster Rovers'!$S$8</f>
         <v/>
       </c>
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="13">
-        <f>'Leyton Orient'!$E$25</f>
+        <f>'Doncaster Rovers'!$E$25</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Plymouth</t>
+          <t>Leyton Orient</t>
         </is>
       </c>
       <c r="B15" s="13">
-        <f>'Plymouth'!$E$24</f>
+        <f>'Leyton Orient'!$E$24</f>
         <v/>
       </c>
       <c r="C15" s="9">
-        <f>'Plymouth'!$S$2</f>
+        <f>'Leyton Orient'!$S$2</f>
         <v/>
       </c>
       <c r="D15" s="9">
-        <f>'Plymouth'!$S$3</f>
+        <f>'Leyton Orient'!$S$3</f>
         <v/>
       </c>
       <c r="E15" s="9">
-        <f>'Plymouth'!$S$4</f>
+        <f>'Leyton Orient'!$S$4</f>
         <v/>
       </c>
       <c r="F15" s="9">
-        <f>'Plymouth'!$S$5</f>
+        <f>'Leyton Orient'!$S$5</f>
         <v/>
       </c>
       <c r="G15" s="9">
-        <f>'Plymouth'!$S$6</f>
+        <f>'Leyton Orient'!$S$6</f>
         <v/>
       </c>
       <c r="H15" s="9">
-        <f>'Plymouth'!$S$7</f>
+        <f>'Leyton Orient'!$S$7</f>
         <v/>
       </c>
       <c r="I15" s="9">
-        <f>'Plymouth'!$S$8</f>
+        <f>'Leyton Orient'!$S$8</f>
         <v/>
       </c>
       <c r="J15" s="6" t="n"/>
       <c r="K15" s="13">
-        <f>'Plymouth'!$E$25</f>
+        <f>'Leyton Orient'!$E$25</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Mansfield</t>
+          <t>Plymouth</t>
         </is>
       </c>
       <c r="B16" s="13">
-        <f>'Mansfield'!$E$24</f>
+        <f>'Plymouth'!$E$24</f>
         <v/>
       </c>
       <c r="C16" s="9">
-        <f>'Mansfield'!$S$2</f>
+        <f>'Plymouth'!$S$2</f>
         <v/>
       </c>
       <c r="D16" s="9">
-        <f>'Mansfield'!$S$3</f>
+        <f>'Plymouth'!$S$3</f>
         <v/>
       </c>
       <c r="E16" s="9">
-        <f>'Mansfield'!$S$4</f>
+        <f>'Plymouth'!$S$4</f>
         <v/>
       </c>
       <c r="F16" s="9">
-        <f>'Mansfield'!$S$5</f>
+        <f>'Plymouth'!$S$5</f>
         <v/>
       </c>
       <c r="G16" s="9">
-        <f>'Mansfield'!$S$6</f>
+        <f>'Plymouth'!$S$6</f>
         <v/>
       </c>
       <c r="H16" s="9">
-        <f>'Mansfield'!$S$7</f>
+        <f>'Plymouth'!$S$7</f>
         <v/>
       </c>
       <c r="I16" s="9">
-        <f>'Mansfield'!$S$8</f>
+        <f>'Plymouth'!$S$8</f>
         <v/>
       </c>
       <c r="J16" s="6" t="n"/>
       <c r="K16" s="13">
-        <f>'Mansfield'!$E$25</f>
+        <f>'Plymouth'!$E$25</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Leicester City</t>
+          <t>Mansfield</t>
         </is>
       </c>
       <c r="B17" s="13">
-        <f>'Leicester City'!$E$24</f>
+        <f>'Mansfield'!$E$24</f>
         <v/>
       </c>
       <c r="C17" s="9">
-        <f>'Leicester City'!$S$2</f>
+        <f>'Mansfield'!$S$2</f>
         <v/>
       </c>
       <c r="D17" s="9">
-        <f>'Leicester City'!$S$3</f>
+        <f>'Mansfield'!$S$3</f>
         <v/>
       </c>
       <c r="E17" s="9">
-        <f>'Leicester City'!$S$4</f>
+        <f>'Mansfield'!$S$4</f>
         <v/>
       </c>
       <c r="F17" s="9">
-        <f>'Leicester City'!$S$5</f>
+        <f>'Mansfield'!$S$5</f>
         <v/>
       </c>
       <c r="G17" s="9">
-        <f>'Leicester City'!$S$6</f>
+        <f>'Mansfield'!$S$6</f>
         <v/>
       </c>
       <c r="H17" s="9">
-        <f>'Leicester City'!$S$7</f>
+        <f>'Mansfield'!$S$7</f>
         <v/>
       </c>
       <c r="I17" s="9">
-        <f>'Leicester City'!$S$8</f>
+        <f>'Mansfield'!$S$8</f>
         <v/>
       </c>
       <c r="J17" s="6" t="n"/>
       <c r="K17" s="13">
-        <f>'Leicester City'!$E$25</f>
+        <f>'Mansfield'!$E$25</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Doncaster Rovers</t>
+          <t>Leicester City</t>
         </is>
       </c>
       <c r="B18" s="13">
-        <f>'Doncaster Rovers'!$E$24</f>
+        <f>'Leicester City'!$E$24</f>
         <v/>
       </c>
       <c r="C18" s="9">
-        <f>'Doncaster Rovers'!$S$2</f>
+        <f>'Leicester City'!$S$2</f>
         <v/>
       </c>
       <c r="D18" s="9">
-        <f>'Doncaster Rovers'!$S$3</f>
+        <f>'Leicester City'!$S$3</f>
         <v/>
       </c>
       <c r="E18" s="9">
-        <f>'Doncaster Rovers'!$S$4</f>
+        <f>'Leicester City'!$S$4</f>
         <v/>
       </c>
       <c r="F18" s="9">
-        <f>'Doncaster Rovers'!$S$5</f>
+        <f>'Leicester City'!$S$5</f>
         <v/>
       </c>
       <c r="G18" s="9">
-        <f>'Doncaster Rovers'!$S$6</f>
+        <f>'Leicester City'!$S$6</f>
         <v/>
       </c>
       <c r="H18" s="9">
-        <f>'Doncaster Rovers'!$S$7</f>
+        <f>'Leicester City'!$S$7</f>
         <v/>
       </c>
       <c r="I18" s="9">
-        <f>'Doncaster Rovers'!$S$8</f>
+        <f>'Leicester City'!$S$8</f>
         <v/>
       </c>
       <c r="J18" s="6" t="n"/>
       <c r="K18" s="13">
-        <f>'Doncaster Rovers'!$E$25</f>
+        <f>'Leicester City'!$E$25</f>
         <v/>
       </c>
     </row>
@@ -3626,39 +3626,39 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Notts County</t>
+          <t>Doncaster Rovers</t>
         </is>
       </c>
       <c r="B3" s="13">
-        <f>'Notts County'!$E$32</f>
+        <f>'Doncaster Rovers'!$E$32</f>
         <v/>
       </c>
       <c r="C3" s="9">
-        <f>'Notts County'!$V$2</f>
+        <f>'Doncaster Rovers'!$V$2</f>
         <v/>
       </c>
       <c r="D3" s="9">
-        <f>'Notts County'!$V$3</f>
+        <f>'Doncaster Rovers'!$V$3</f>
         <v/>
       </c>
       <c r="E3" s="9">
-        <f>'Notts County'!$V$4</f>
+        <f>'Doncaster Rovers'!$V$4</f>
         <v/>
       </c>
       <c r="F3" s="9">
-        <f>'Notts County'!$V$5</f>
+        <f>'Doncaster Rovers'!$V$5</f>
         <v/>
       </c>
       <c r="G3" s="9">
-        <f>'Notts County'!$V$6</f>
+        <f>'Doncaster Rovers'!$V$6</f>
         <v/>
       </c>
       <c r="H3" s="9">
-        <f>'Notts County'!$V$7</f>
+        <f>'Doncaster Rovers'!$V$7</f>
         <v/>
       </c>
       <c r="I3" s="9">
-        <f>'Notts County'!$V$8</f>
+        <f>'Doncaster Rovers'!$V$8</f>
         <v/>
       </c>
       <c r="J3" s="6" t="n"/>
@@ -3666,39 +3666,39 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Doncaster Rovers</t>
+          <t>Notts County</t>
         </is>
       </c>
       <c r="B4" s="13">
-        <f>'Doncaster Rovers'!$E$32</f>
+        <f>'Notts County'!$E$32</f>
         <v/>
       </c>
       <c r="C4" s="9">
-        <f>'Doncaster Rovers'!$V$2</f>
+        <f>'Notts County'!$V$2</f>
         <v/>
       </c>
       <c r="D4" s="9">
-        <f>'Doncaster Rovers'!$V$3</f>
+        <f>'Notts County'!$V$3</f>
         <v/>
       </c>
       <c r="E4" s="9">
-        <f>'Doncaster Rovers'!$V$4</f>
+        <f>'Notts County'!$V$4</f>
         <v/>
       </c>
       <c r="F4" s="9">
-        <f>'Doncaster Rovers'!$V$5</f>
+        <f>'Notts County'!$V$5</f>
         <v/>
       </c>
       <c r="G4" s="9">
-        <f>'Doncaster Rovers'!$V$6</f>
+        <f>'Notts County'!$V$6</f>
         <v/>
       </c>
       <c r="H4" s="9">
-        <f>'Doncaster Rovers'!$V$7</f>
+        <f>'Notts County'!$V$7</f>
         <v/>
       </c>
       <c r="I4" s="9">
-        <f>'Doncaster Rovers'!$V$8</f>
+        <f>'Notts County'!$V$8</f>
         <v/>
       </c>
       <c r="J4" s="6" t="n"/>
@@ -4570,12 +4570,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
     <col width="31" customWidth="1" min="5" max="5"/>
     <col width="31" customWidth="1" min="6" max="6"/>
@@ -4652,467 +4652,173 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Reading</t>
+          <t>Stockport County</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>Notts County</t>
+          <t>Peterborough United</t>
         </is>
       </c>
       <c r="D2" s="9" t="n">
-        <v>0.66</v>
+        <v>1.47</v>
       </c>
       <c r="E2" s="9" t="n">
-        <v>1.28</v>
+        <v>0.38</v>
       </c>
       <c r="F2" s="9" t="n">
-        <v>0.43</v>
+        <v>0.19</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>1.51</v>
+        <v>1.66</v>
       </c>
       <c r="H2" s="9" t="n">
-        <v>2.76</v>
+        <v>3.5</v>
       </c>
       <c r="I2" s="9" t="n">
-        <v>0.58</v>
+        <v>0.34</v>
       </c>
       <c r="J2" s="9" t="n">
-        <v>-0.25</v>
+        <v>-0.09</v>
       </c>
       <c r="K2" s="9" t="n">
-        <v>3.09</v>
+        <v>3.75</v>
       </c>
       <c r="L2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Oxford United</t>
+          <t>Plymouth</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>Cambridge</t>
+          <t>Burton Albion</t>
         </is>
       </c>
       <c r="D3" s="10" t="n">
-        <v>0.37</v>
+        <v>0.95</v>
       </c>
       <c r="E3" s="10" t="n">
-        <v>-0.1</v>
+        <v>-0.13</v>
       </c>
       <c r="F3" s="10" t="n">
-        <v>-0.24</v>
+        <v>-0.28</v>
       </c>
       <c r="G3" s="10" t="n">
-        <v>0.51</v>
+        <v>1.1</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>2.68</v>
+        <v>2.97</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>0.38</v>
+        <v>-0.05</v>
       </c>
       <c r="J3" s="10" t="n">
-        <v>0.16</v>
+        <v>-0.34</v>
       </c>
       <c r="K3" s="10" t="n">
-        <v>3.22</v>
+        <v>2.58</v>
       </c>
       <c r="L3" s="8" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Luton</t>
+          <t>Cambridge</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Bradford City</t>
+          <t>AFC Wimbledon</t>
         </is>
       </c>
       <c r="D4" s="9" t="n">
-        <v>0.43</v>
+        <v>0.67</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>-0.02</v>
+        <v>-0.24</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>-0.09</v>
+        <v>-0.16</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>0.5</v>
+        <v>0.59</v>
       </c>
       <c r="H4" s="9" t="n">
-        <v>2.71</v>
+        <v>2.55</v>
       </c>
       <c r="I4" s="9" t="n">
-        <v>-0.4</v>
+        <v>0.16</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>-0.64</v>
+        <v>-0.24</v>
       </c>
       <c r="K4" s="9" t="n">
-        <v>1.67</v>
+        <v>2.47</v>
       </c>
       <c r="L4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Wigan Athletic</t>
+          <t>Wycombe Wanderers</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Wycombe Wanderers</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="D5" s="10" t="n">
         <v>0.02</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>0.14</v>
+        <v>-0.01</v>
       </c>
       <c r="F5" s="10" t="n">
-        <v>-0.01</v>
+        <v>1.25</v>
       </c>
       <c r="G5" s="10" t="n">
-        <v>0.17</v>
+        <v>-1.24</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>2.86</v>
+        <v>2.96</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>0.65</v>
+        <v>0.05</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>0.05</v>
+        <v>0.55</v>
       </c>
       <c r="K5" s="10" t="n">
         <v>3.56</v>
       </c>
       <c r="L5" s="8" t="inlineStr"/>
     </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Barnsley</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Leicester City</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="n">
-        <v>-0.46</v>
-      </c>
-      <c r="E6" s="9" t="n">
-        <v>-0.02</v>
-      </c>
-      <c r="F6" s="9" t="n">
-        <v>-0.52</v>
-      </c>
-      <c r="G6" s="9" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="H6" s="9" t="n">
-        <v>3.31</v>
-      </c>
-      <c r="I6" s="9" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="J6" s="9" t="n">
-        <v>-0.07000000000000001</v>
-      </c>
-      <c r="K6" s="9" t="n">
-        <v>3.37</v>
-      </c>
-      <c r="L6" s="6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>Peterborough United</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Doncaster Rovers</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="E7" s="10" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="F7" s="10" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="G7" s="10" t="n">
-        <v>-0.12</v>
-      </c>
-      <c r="H7" s="10" t="n">
-        <v>3.08</v>
-      </c>
-      <c r="I7" s="10" t="n">
-        <v>-0.18</v>
-      </c>
-      <c r="J7" s="10" t="n">
-        <v>-0.09</v>
-      </c>
-      <c r="K7" s="10" t="n">
-        <v>2.81</v>
-      </c>
-      <c r="L7" s="8" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Burton Albion</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Mansfield</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="E8" s="9" t="n">
-        <v>-0.28</v>
-      </c>
-      <c r="F8" s="9" t="n">
-        <v>-0.07000000000000001</v>
-      </c>
-      <c r="G8" s="9" t="n">
-        <v>-0.19</v>
-      </c>
-      <c r="H8" s="9" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="I8" s="9" t="n">
-        <v>-0.34</v>
-      </c>
-      <c r="J8" s="9" t="n">
-        <v>-0.06</v>
-      </c>
-      <c r="K8" s="9" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="L8" s="6" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Sheffield Wednesday</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Stockport County</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="n">
-        <v>-0.28</v>
-      </c>
-      <c r="E9" s="10" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="F9" s="10" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="G9" s="10" t="n">
-        <v>-0.33</v>
-      </c>
-      <c r="H9" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="I9" s="10" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="J9" s="10" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="K9" s="10" t="n">
-        <v>3.82</v>
-      </c>
-      <c r="L9" s="8" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Leyton Orient</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>Stevenage</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="E10" s="9" t="n">
-        <v>-0.65</v>
-      </c>
-      <c r="F10" s="9" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G10" s="9" t="n">
-        <v>-0.59</v>
-      </c>
-      <c r="H10" s="9" t="n">
-        <v>2.46</v>
-      </c>
-      <c r="I10" s="9" t="n">
-        <v>-0.02</v>
-      </c>
-      <c r="J10" s="9" t="n">
-        <v>-0.41</v>
-      </c>
-      <c r="K10" s="9" t="n">
-        <v>2.03</v>
-      </c>
-      <c r="L10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Blackpool</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Plymouth</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="n">
-        <v>-0.04</v>
-      </c>
-      <c r="E11" s="10" t="n">
-        <v>-0.7</v>
-      </c>
-      <c r="F11" s="10" t="n">
-        <v>-0.13</v>
-      </c>
-      <c r="G11" s="10" t="n">
-        <v>-0.61</v>
-      </c>
-      <c r="H11" s="10" t="n">
-        <v>3.02</v>
-      </c>
-      <c r="I11" s="10" t="n">
-        <v>1.09</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>-0.05</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>4.06</v>
-      </c>
-      <c r="L11" s="8" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Bromley</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>Huddersfield Town</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="n">
-        <v>-1.01</v>
-      </c>
-      <c r="E12" s="9" t="n">
-        <v>-0.53</v>
-      </c>
-      <c r="F12" s="9" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="G12" s="9" t="n">
-        <v>-1.86</v>
-      </c>
-      <c r="H12" s="9" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="I12" s="9" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="J12" s="9" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="K12" s="9" t="n">
-        <v>3.14</v>
-      </c>
-      <c r="L12" s="6" t="inlineStr"/>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="G2:G12">
+  <conditionalFormatting sqref="G2:G5">
     <cfRule type="dataBar" priority="1">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -5131,7 +4837,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K12">
+  <conditionalFormatting sqref="K2:K5">
     <cfRule type="dataBar" priority="3">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -5433,13 +5139,13 @@
         <v>-0.6899999999999999</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>-1.11</v>
+        <v>-1.07</v>
       </c>
       <c r="P3" s="10" t="n">
         <v>-0.65</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>-1.09</v>
+        <v>-1.07</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -5521,7 +5227,7 @@
         <v>-0.49</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.27</v>
+        <v>-0.26</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -5594,7 +5300,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="N5" s="10" t="n">
-        <v>0.44</v>
+        <v>0.43</v>
       </c>
       <c r="O5" s="10" t="n">
         <v>-0.35</v>
@@ -5603,7 +5309,7 @@
         <v>-0.26</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>-0.29</v>
+        <v>-0.28</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -5758,16 +5464,16 @@
         <v>0.09</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>-0.28</v>
+        <v>-0.32</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>1.07</v>
+        <v>1</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.28</v>
+        <v>-0.29</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>-0.13</v>
+        <v>-0.14</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -5846,7 +5552,7 @@
         <v>-0.68</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>-0.21</v>
+        <v>-0.22</v>
       </c>
       <c r="Q8" s="9" t="n">
         <v>-0.07000000000000001</v>
@@ -5928,10 +5634,10 @@
         <v>-0.64</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>-0.13</v>
+        <v>-0.14</v>
       </c>
       <c r="Q9" s="10" t="n">
-        <v>0.01</v>
+        <v>-0</v>
       </c>
       <c r="R9" s="10">
         <f>(H9-I9)-(F9-G9)</f>
@@ -6786,16 +6492,16 @@
         <v>0.2</v>
       </c>
       <c r="N3" s="10" t="n">
-        <v>-0.57</v>
+        <v>-0.61</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>-0.04</v>
+        <v>-0.11</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>-0.59</v>
+        <v>-0.61</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>0.26</v>
+        <v>0.23</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -6874,10 +6580,10 @@
         <v>-0.67</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.18</v>
+        <v>-0.19</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.05</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -6956,10 +6662,10 @@
         <v>0.68</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>-0.15</v>
+        <v>-0.16</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -7038,10 +6744,10 @@
         <v>1.14</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -7120,10 +6826,10 @@
         <v>-1.19</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.06</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -7202,10 +6908,10 @@
         <v>0.95</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>-0.05</v>
+        <v>-0.06</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -8060,16 +7766,16 @@
         <v>0.83</v>
       </c>
       <c r="N3" s="10" t="n">
-        <v>1.08</v>
+        <v>1.03</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>1.54</v>
+        <v>1.51</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>1.11</v>
+        <v>1.09</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -8142,16 +7848,16 @@
         <v>0.66</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>1.16</v>
+        <v>1.09</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>0.36</v>
+        <v>0.32</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>1.12</v>
+        <v>1.09</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>0.62</v>
+        <v>0.6</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -8230,10 +7936,10 @@
         <v>0.9</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>1.05</v>
+        <v>1.02</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.67</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -8306,16 +8012,16 @@
         <v>0.93</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>-0.31</v>
+        <v>-0.3</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>1.12</v>
+        <v>1.15</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.78</v>
+        <v>0.76</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -8394,10 +8100,10 @@
         <v>0.67</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.47</v>
+        <v>0.45</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -8476,7 +8182,7 @@
         <v>1.55</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.11</v>
+        <v>0.09</v>
       </c>
       <c r="Q8" s="9" t="n">
         <v>1.02</v>
@@ -9252,16 +8958,16 @@
         <v>0.15</v>
       </c>
       <c r="N2" s="9" t="n">
-        <v>0.42</v>
+        <v>0.35</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>0.16</v>
+        <v>0.12</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>0.42</v>
+        <v>0.35</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>0.16</v>
+        <v>0.12</v>
       </c>
       <c r="R2" s="9">
         <f>(H2-I2)-(F2-G2)</f>
@@ -9334,16 +9040,16 @@
         <v>0.14</v>
       </c>
       <c r="N3" s="10" t="n">
-        <v>-0.92</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>-0.36</v>
+        <v>-0.41</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>-0.25</v>
+        <v>-0.3</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>-0.1</v>
+        <v>-0.14</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -9422,10 +9128,10 @@
         <v>-0.29</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.32</v>
+        <v>-0.36</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.16</v>
+        <v>-0.19</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -9504,10 +9210,10 @@
         <v>0.09</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>-0.16</v>
+        <v>-0.19</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>-0.1</v>
+        <v>-0.12</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -9583,13 +9289,13 @@
         <v>-0.57</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>-0.58</v>
+        <v>-0.59</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.24</v>
+        <v>-0.26</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>-0.2</v>
+        <v>-0.21</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -9662,16 +9368,16 @@
         <v>-0.2</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.53</v>
       </c>
       <c r="O7" s="10" t="n">
         <v>-0.85</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.3</v>
+        <v>-0.31</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>-0.3</v>
+        <v>-0.32</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -9753,7 +9459,7 @@
         <v>-0.5</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.43</v>
+        <v>-0.44</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -10690,16 +10396,16 @@
         <v>0.54</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>0.5</v>
+        <v>0.48</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>2.44</v>
+        <v>2.4</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.11</v>
+        <v>-0.12</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>0.45</v>
+        <v>0.43</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -10781,7 +10487,7 @@
         <v>-0.38</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>0.53</v>
+        <v>0.52</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -10860,10 +10566,10 @@
         <v>0.2</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.48</v>
+        <v>-0.49</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.47</v>
+        <v>0.46</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -10942,7 +10648,7 @@
         <v>-0.98</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.51</v>
+        <v>-0.52</v>
       </c>
       <c r="Q7" s="10" t="n">
         <v>0.22</v>
@@ -13074,13 +12780,13 @@
         <v>-0.19</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>-0.8</v>
+        <v>-0.77</v>
       </c>
       <c r="O4" s="9" t="n">
         <v>0.66</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.41</v>
+        <v>-0.4</v>
       </c>
       <c r="Q4" s="9" t="n">
         <v>-0.1</v>
@@ -13387,31 +13093,31 @@
         <v>0.85</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>1.82</v>
+        <v>1.87</v>
       </c>
       <c r="J8" s="9" t="n">
         <v>-0.51</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>0.48</v>
+        <v>0.53</v>
       </c>
       <c r="L8" s="9" t="n">
         <v>-0.31</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="N8" s="9" t="n">
         <v>-0.6</v>
       </c>
       <c r="O8" s="9" t="n">
-        <v>0.64</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>-0.42</v>
+        <v>-0.41</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -13422,16 +13128,16 @@
         <v/>
       </c>
       <c r="T8" s="9" t="n">
-        <v>0.74</v>
+        <v>0.72</v>
       </c>
       <c r="U8" s="9" t="n">
         <v>1.39</v>
       </c>
       <c r="V8" s="9" t="n">
-        <v>-0.65</v>
+        <v>-0.67</v>
       </c>
       <c r="W8" s="9" t="n">
-        <v>7.36</v>
+        <v>7.34</v>
       </c>
       <c r="X8" s="9" t="n">
         <v>8.84</v>
@@ -13751,16 +13457,16 @@
         <v>6</v>
       </c>
       <c r="E36" s="19" t="n">
-        <v>-0.19</v>
+        <v>-0.2</v>
       </c>
       <c r="F36" s="19" t="n">
         <v>-0.39</v>
       </c>
       <c r="G36" s="19" t="n">
-        <v>-0.03</v>
+        <v>-0.02</v>
       </c>
       <c r="H36" s="19" t="n">
-        <v>-0.15</v>
+        <v>-0.12</v>
       </c>
     </row>
     <row r="37">
@@ -14512,7 +14218,7 @@
         <v>0.3</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="O6" s="9" t="n">
         <v>1.53</v>
@@ -14597,13 +14303,13 @@
         <v>-0.03</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>-0.27</v>
+        <v>-0.24</v>
       </c>
       <c r="P7" s="10" t="n">
         <v>-0.06</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -14685,7 +14391,7 @@
         <v>-0.1</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.02</v>
+        <v>-0.01</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -15461,13 +15167,13 @@
         <v>-0.11</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>-0.02</v>
+        <v>-0.03</v>
       </c>
       <c r="P2" s="9" t="n">
         <v>-0.11</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>-0.02</v>
+        <v>-0.03</v>
       </c>
       <c r="R2" s="9">
         <f>(H2-I2)-(F2-G2)</f>
@@ -15704,13 +15410,13 @@
         <v>-0.5</v>
       </c>
       <c r="N5" s="10" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="O5" s="10" t="n">
+        <v>-0.51</v>
+      </c>
+      <c r="P5" s="10" t="n">
         <v>-0.01</v>
-      </c>
-      <c r="O5" s="10" t="n">
-        <v>-0.52</v>
-      </c>
-      <c r="P5" s="10" t="n">
-        <v>-0.02</v>
       </c>
       <c r="Q5" s="10" t="n">
         <v>-0.58</v>
@@ -15792,7 +15498,7 @@
         <v>1.22</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="Q6" s="9" t="n">
         <v>-0.22</v>
@@ -15932,34 +15638,34 @@
         <v>1.6</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>1.1</v>
+        <v>1.51</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>1.27</v>
+        <v>1.51</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>-0.38</v>
+        <v>0.03</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>-0.33</v>
+        <v>-0.09</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>0.22</v>
+        <v>0.29</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>-0.3</v>
+        <v>-0.26</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>-0.21</v>
+        <v>0.2</v>
       </c>
       <c r="O8" s="9" t="n">
-        <v>-0.4</v>
+        <v>-0.16</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.4</v>
+        <v>0.47</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.3</v>
+        <v>-0.26</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -15970,16 +15676,16 @@
         <v/>
       </c>
       <c r="T8" s="9" t="n">
-        <v>1.24</v>
+        <v>1.38</v>
       </c>
       <c r="U8" s="9" t="n">
         <v>1.31</v>
       </c>
       <c r="V8" s="9" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="W8" s="9" t="n">
-        <v>11.59</v>
+        <v>11.73</v>
       </c>
       <c r="X8" s="9" t="n">
         <v>9.630000000000001</v>
@@ -16327,16 +16033,16 @@
         <v>5</v>
       </c>
       <c r="E37" s="19" t="n">
-        <v>0.5</v>
+        <v>0.54</v>
       </c>
       <c r="F37" s="19" t="n">
-        <v>0.23</v>
+        <v>0.29</v>
       </c>
       <c r="G37" s="19" t="n">
-        <v>-0.36</v>
+        <v>-0.2</v>
       </c>
       <c r="H37" s="19" t="n">
-        <v>-0.44</v>
+        <v>-0.12</v>
       </c>
     </row>
     <row r="38">
@@ -16355,16 +16061,16 @@
         <v>9</v>
       </c>
       <c r="E38" s="21" t="n">
-        <v>0.44</v>
+        <v>0.47</v>
       </c>
       <c r="F38" s="21" t="n">
         <v>0.2</v>
       </c>
       <c r="G38" s="21" t="n">
-        <v>-0.09</v>
+        <v>-0</v>
       </c>
       <c r="H38" s="21" t="n">
-        <v>-0.62</v>
+        <v>-0.17</v>
       </c>
     </row>
   </sheetData>
@@ -17060,13 +16766,13 @@
         <v>0.08</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>0.09</v>
+        <v>0.12</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>0.49</v>
+        <v>0.5</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="Q6" s="9" t="n">
         <v>0.06</v>
@@ -17145,10 +16851,10 @@
         <v>-0.37</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>-0.33</v>
+        <v>-0.34</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="Q7" s="10" t="n">
         <v>-0</v>
@@ -17230,7 +16936,7 @@
         <v>-0.37</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.36</v>
+        <v>0.37</v>
       </c>
       <c r="Q8" s="9" t="n">
         <v>0.01</v>
@@ -18006,13 +17712,13 @@
         <v>1.12</v>
       </c>
       <c r="N2" s="9" t="n">
-        <v>-0.51</v>
+        <v>-0.48</v>
       </c>
       <c r="O2" s="9" t="n">
         <v>1.21</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>-0.51</v>
+        <v>-0.48</v>
       </c>
       <c r="Q2" s="9" t="n">
         <v>1.21</v>
@@ -18088,13 +17794,13 @@
         <v>0.49</v>
       </c>
       <c r="N3" s="10" t="n">
-        <v>-0.79</v>
+        <v>-0.8</v>
       </c>
       <c r="O3" s="10" t="n">
         <v>0.2</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>-0.65</v>
+        <v>-0.64</v>
       </c>
       <c r="Q3" s="10" t="n">
         <v>0.71</v>
@@ -18176,7 +17882,7 @@
         <v>-1.1</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.51</v>
+        <v>-0.5</v>
       </c>
       <c r="Q4" s="9" t="n">
         <v>0.1</v>
@@ -18258,7 +17964,7 @@
         <v>0.02</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>-0.48</v>
+        <v>-0.47</v>
       </c>
       <c r="Q5" s="10" t="n">
         <v>0.08</v>
@@ -18340,7 +18046,7 @@
         <v>1.37</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.64</v>
+        <v>-0.63</v>
       </c>
       <c r="Q6" s="9" t="n">
         <v>0.34</v>
@@ -18416,10 +18122,10 @@
         <v>0.3</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.03</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>0.12</v>
+        <v>0.09</v>
       </c>
       <c r="P7" s="10" t="n">
         <v>-0.52</v>
@@ -18504,7 +18210,7 @@
         <v>-0.35</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>-0.35</v>
+        <v>-0.36</v>
       </c>
       <c r="Q8" s="9" t="n">
         <v>0.04</v>
@@ -19280,16 +18986,16 @@
         <v>1.4</v>
       </c>
       <c r="N2" s="9" t="n">
-        <v>0.03</v>
+        <v>-0</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>1.12</v>
+        <v>1.08</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>0.03</v>
+        <v>-0</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>1.12</v>
+        <v>1.08</v>
       </c>
       <c r="R2" s="9">
         <f>(H2-I2)-(F2-G2)</f>
@@ -19368,10 +19074,10 @@
         <v>-0.2</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>-0.03</v>
+        <v>-0.05</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>0.46</v>
+        <v>0.44</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -19450,10 +19156,10 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.41</v>
+        <v>-0.42</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>0.62</v>
+        <v>0.61</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -19532,10 +19238,10 @@
         <v>-0.54</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>-0.29</v>
+        <v>-0.3</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -19614,10 +19320,10 @@
         <v>0.43</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.31</v>
+        <v>-0.32</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.35</v>
+        <v>0.34</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -19696,7 +19402,7 @@
         <v>-0.29</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.37</v>
+        <v>-0.38</v>
       </c>
       <c r="Q7" s="10" t="n">
         <v>0.24</v>
@@ -20557,13 +20263,13 @@
         <v>0.55</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>-0.59</v>
+        <v>-0.55</v>
       </c>
       <c r="P2" s="9" t="n">
         <v>0.55</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>-0.59</v>
+        <v>-0.55</v>
       </c>
       <c r="R2" s="9">
         <f>(H2-I2)-(F2-G2)</f>
@@ -20636,16 +20342,16 @@
         <v>0.11</v>
       </c>
       <c r="N3" s="10" t="n">
-        <v>0.33</v>
+        <v>0.36</v>
       </c>
       <c r="O3" s="10" t="n">
         <v>-0.35</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>0.44</v>
+        <v>0.46</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>-0.47</v>
+        <v>-0.45</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -20721,13 +20427,13 @@
         <v>-0.25</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>0.35</v>
+        <v>0.34</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.2</v>
+        <v>-0.19</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -20800,10 +20506,10 @@
         <v>-0.02</v>
       </c>
       <c r="N5" s="10" t="n">
-        <v>-0.17</v>
+        <v>-0.21</v>
       </c>
       <c r="O5" s="10" t="n">
-        <v>-1.03</v>
+        <v>-1.06</v>
       </c>
       <c r="P5" s="10" t="n">
         <v>0.11</v>
@@ -20888,7 +20594,7 @@
         <v>-0.22</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="Q6" s="9" t="n">
         <v>-0.37</v>
@@ -20970,7 +20676,7 @@
         <v>0.27</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q7" s="10" t="n">
         <v>-0.26</v>
@@ -21055,7 +20761,7 @@
         <v>-0.18</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.26</v>
+        <v>-0.27</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -21828,16 +21534,16 @@
         <v>-0.09</v>
       </c>
       <c r="N2" s="9" t="n">
-        <v>0.22</v>
+        <v>0.18</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>-0.31</v>
+        <v>-0.38</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>0.22</v>
+        <v>0.18</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>-0.31</v>
+        <v>-0.38</v>
       </c>
       <c r="R2" s="9">
         <f>(H2-I2)-(F2-G2)</f>
@@ -21910,16 +21616,16 @@
         <v>-0.06</v>
       </c>
       <c r="N3" s="10" t="n">
-        <v>-0.17</v>
+        <v>-0.24</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>-0.06</v>
+        <v>-0.1</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>0.02</v>
+        <v>-0.03</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>-0.19</v>
+        <v>-0.24</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -21998,10 +21704,10 @@
         <v>-0.01</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>0.18</v>
+        <v>0.15</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.13</v>
+        <v>-0.16</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -22077,13 +21783,13 @@
         <v>0.62</v>
       </c>
       <c r="O5" s="10" t="n">
-        <v>0.88</v>
+        <v>0.92</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>0.29</v>
+        <v>0.26</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -22162,10 +21868,10 @@
         <v>-0.14</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -22244,10 +21950,10 @@
         <v>-0.66</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.09</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>-0.05</v>
+        <v>-0.06</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -22302,25 +22008,25 @@
         <v>1.36</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>1.82</v>
+        <v>1.87</v>
       </c>
       <c r="I8" s="9" t="n">
         <v>0.85</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>0.48</v>
+        <v>0.53</v>
       </c>
       <c r="K8" s="9" t="n">
         <v>-0.51</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>-0.06</v>
+        <v>-0.05</v>
       </c>
       <c r="M8" s="9" t="n">
         <v>0.02</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>0.6</v>
+        <v>0.65</v>
       </c>
       <c r="O8" s="9" t="n">
         <v>-0.23</v>
@@ -22340,16 +22046,16 @@
         <v/>
       </c>
       <c r="T8" s="9" t="n">
-        <v>2.04</v>
+        <v>2.06</v>
       </c>
       <c r="U8" s="9" t="n">
         <v>1.36</v>
       </c>
       <c r="V8" s="9" t="n">
-        <v>0.68</v>
+        <v>0.71</v>
       </c>
       <c r="W8" s="9" t="n">
-        <v>8.74</v>
+        <v>8.77</v>
       </c>
       <c r="X8" s="9" t="n">
         <v>8.82</v>
@@ -22697,16 +22403,16 @@
         <v>10</v>
       </c>
       <c r="E37" s="19" t="n">
-        <v>-0.22</v>
+        <v>-0.21</v>
       </c>
       <c r="F37" s="19" t="n">
         <v>-0.19</v>
       </c>
       <c r="G37" s="19" t="n">
-        <v>0.09</v>
+        <v>0.11</v>
       </c>
       <c r="H37" s="19" t="n">
-        <v>-0.21</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="38">
@@ -22725,7 +22431,7 @@
         <v>13</v>
       </c>
       <c r="E38" s="21" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.06</v>
       </c>
       <c r="F38" s="21" t="n">
         <v>-0.03</v>
@@ -23512,13 +23218,13 @@
         <v>0.25</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>-0.42</v>
+        <v>-0.49</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>-0.18</v>
+        <v>-0.22</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.31</v>
+        <v>0.29</v>
       </c>
       <c r="Q7" s="10" t="n">
         <v>0.19</v>
@@ -23600,7 +23306,7 @@
         <v>0.26</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="Q8" s="9" t="n">
         <v>0.18</v>
@@ -23682,10 +23388,10 @@
         <v>0.22</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.08</v>
       </c>
       <c r="Q9" s="10" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="R9" s="10">
         <f>(H9-I9)-(F9-G9)</f>
@@ -24622,13 +24328,13 @@
         <v>-0.62</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="O4" s="9" t="n">
         <v>-0.83</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>0.61</v>
+        <v>0.6</v>
       </c>
       <c r="Q4" s="9" t="n">
         <v>-0.41</v>
@@ -24704,16 +24410,16 @@
         <v>-0.55</v>
       </c>
       <c r="N5" s="10" t="n">
-        <v>-0.1</v>
+        <v>-0.14</v>
       </c>
       <c r="O5" s="10" t="n">
-        <v>-0.61</v>
+        <v>-0.68</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>0.43</v>
+        <v>0.42</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>-0.46</v>
+        <v>-0.48</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -24792,10 +24498,10 @@
         <v>-0.61</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>-0.49</v>
+        <v>-0.5</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -24874,10 +24580,10 @@
         <v>-0.53</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>-0.5</v>
+        <v>-0.51</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -24932,34 +24638,34 @@
         <v>1.71</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>0.59</v>
+        <v>0.58</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>2.62</v>
+        <v>2.44</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>-0.46</v>
+        <v>-0.47</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>0.91</v>
+        <v>0.73</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>-0.08</v>
+        <v>-0.09</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>-0.27</v>
+        <v>-0.3</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>-0.13</v>
+        <v>-0.14</v>
       </c>
       <c r="O8" s="9" t="n">
-        <v>-0.03</v>
+        <v>-0.21</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.41</v>
+        <v>-0.45</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -24970,16 +24676,16 @@
         <v/>
       </c>
       <c r="T8" s="9" t="n">
-        <v>0.32</v>
+        <v>0.35</v>
       </c>
       <c r="U8" s="9" t="n">
         <v>0.9399999999999999</v>
       </c>
       <c r="V8" s="9" t="n">
-        <v>-0.62</v>
+        <v>-0.58</v>
       </c>
       <c r="W8" s="9" t="n">
-        <v>9.6</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="X8" s="9" t="n">
         <v>7.51</v>
@@ -25327,13 +25033,13 @@
         <v>6</v>
       </c>
       <c r="E37" s="19" t="n">
-        <v>-0.19</v>
+        <v>-0.14</v>
       </c>
       <c r="F37" s="19" t="n">
         <v>-0.08</v>
       </c>
       <c r="G37" s="19" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.12</v>
       </c>
       <c r="H37" s="19" t="n">
         <v>-0.02</v>
@@ -25355,13 +25061,13 @@
         <v>9</v>
       </c>
       <c r="E38" s="21" t="n">
-        <v>0.43</v>
+        <v>0.46</v>
       </c>
       <c r="F38" s="21" t="n">
         <v>0.18</v>
       </c>
       <c r="G38" s="21" t="n">
-        <v>-0.25</v>
+        <v>-0.28</v>
       </c>
       <c r="H38" s="21" t="n">
         <v>-0.27</v>
@@ -25871,102 +25577,102 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Blackpool</t>
+          <t>Doncaster Rovers</t>
         </is>
       </c>
       <c r="B7" s="8">
-        <f>'Blackpool'!$E$11</f>
+        <f>'Doncaster Rovers'!$E$11</f>
         <v/>
       </c>
       <c r="C7" s="10">
-        <f>'Blackpool'!$E$14</f>
+        <f>'Doncaster Rovers'!$E$14</f>
         <v/>
       </c>
       <c r="D7" s="10">
-        <f>'Blackpool'!$E$16</f>
+        <f>'Doncaster Rovers'!$E$16</f>
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>'Blackpool'!$E$18</f>
+        <f>'Doncaster Rovers'!$E$18</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>'Blackpool'!$E$20</f>
+        <f>'Doncaster Rovers'!$E$20</f>
         <v/>
       </c>
       <c r="G7" s="10">
-        <f>'Blackpool'!$E$22</f>
+        <f>'Doncaster Rovers'!$E$22</f>
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>'Blackpool'!$E$26</f>
+        <f>'Doncaster Rovers'!$E$26</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>'Blackpool'!$E$27</f>
+        <f>'Doncaster Rovers'!$E$27</f>
         <v/>
       </c>
       <c r="J7" s="10">
-        <f>'Blackpool'!$E$30</f>
+        <f>'Doncaster Rovers'!$E$30</f>
         <v/>
       </c>
       <c r="K7" s="10">
-        <f>'Blackpool'!$E$31</f>
+        <f>'Doncaster Rovers'!$E$31</f>
         <v/>
       </c>
       <c r="L7" s="10">
-        <f>'Blackpool'!$E$32</f>
+        <f>'Doncaster Rovers'!$E$32</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Doncaster Rovers</t>
+          <t>Blackpool</t>
         </is>
       </c>
       <c r="B8" s="6">
-        <f>'Doncaster Rovers'!$E$11</f>
+        <f>'Blackpool'!$E$11</f>
         <v/>
       </c>
       <c r="C8" s="9">
-        <f>'Doncaster Rovers'!$E$14</f>
+        <f>'Blackpool'!$E$14</f>
         <v/>
       </c>
       <c r="D8" s="9">
-        <f>'Doncaster Rovers'!$E$16</f>
+        <f>'Blackpool'!$E$16</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>'Doncaster Rovers'!$E$18</f>
+        <f>'Blackpool'!$E$18</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>'Doncaster Rovers'!$E$20</f>
+        <f>'Blackpool'!$E$20</f>
         <v/>
       </c>
       <c r="G8" s="9">
-        <f>'Doncaster Rovers'!$E$22</f>
+        <f>'Blackpool'!$E$22</f>
         <v/>
       </c>
       <c r="H8" s="9">
-        <f>'Doncaster Rovers'!$E$26</f>
+        <f>'Blackpool'!$E$26</f>
         <v/>
       </c>
       <c r="I8" s="9">
-        <f>'Doncaster Rovers'!$E$27</f>
+        <f>'Blackpool'!$E$27</f>
         <v/>
       </c>
       <c r="J8" s="9">
-        <f>'Doncaster Rovers'!$E$30</f>
+        <f>'Blackpool'!$E$30</f>
         <v/>
       </c>
       <c r="K8" s="9">
-        <f>'Doncaster Rovers'!$E$31</f>
+        <f>'Blackpool'!$E$31</f>
         <v/>
       </c>
       <c r="L8" s="9">
-        <f>'Doncaster Rovers'!$E$32</f>
+        <f>'Blackpool'!$E$32</f>
         <v/>
       </c>
     </row>
@@ -26177,102 +25883,102 @@
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Wycombe Wanderers</t>
+          <t>Peterborough United</t>
         </is>
       </c>
       <c r="B13" s="8">
-        <f>'Wycombe Wanderers'!$E$11</f>
+        <f>'Peterborough United'!$E$11</f>
         <v/>
       </c>
       <c r="C13" s="10">
-        <f>'Wycombe Wanderers'!$E$14</f>
+        <f>'Peterborough United'!$E$14</f>
         <v/>
       </c>
       <c r="D13" s="10">
-        <f>'Wycombe Wanderers'!$E$16</f>
+        <f>'Peterborough United'!$E$16</f>
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>'Wycombe Wanderers'!$E$18</f>
+        <f>'Peterborough United'!$E$18</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>'Wycombe Wanderers'!$E$20</f>
+        <f>'Peterborough United'!$E$20</f>
         <v/>
       </c>
       <c r="G13" s="10">
-        <f>'Wycombe Wanderers'!$E$22</f>
+        <f>'Peterborough United'!$E$22</f>
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>'Wycombe Wanderers'!$E$26</f>
+        <f>'Peterborough United'!$E$26</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>'Wycombe Wanderers'!$E$27</f>
+        <f>'Peterborough United'!$E$27</f>
         <v/>
       </c>
       <c r="J13" s="10">
-        <f>'Wycombe Wanderers'!$E$30</f>
+        <f>'Peterborough United'!$E$30</f>
         <v/>
       </c>
       <c r="K13" s="10">
-        <f>'Wycombe Wanderers'!$E$31</f>
+        <f>'Peterborough United'!$E$31</f>
         <v/>
       </c>
       <c r="L13" s="10">
-        <f>'Wycombe Wanderers'!$E$32</f>
+        <f>'Peterborough United'!$E$32</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Peterborough United</t>
+          <t>Wycombe Wanderers</t>
         </is>
       </c>
       <c r="B14" s="6">
-        <f>'Peterborough United'!$E$11</f>
+        <f>'Wycombe Wanderers'!$E$11</f>
         <v/>
       </c>
       <c r="C14" s="9">
-        <f>'Peterborough United'!$E$14</f>
+        <f>'Wycombe Wanderers'!$E$14</f>
         <v/>
       </c>
       <c r="D14" s="9">
-        <f>'Peterborough United'!$E$16</f>
+        <f>'Wycombe Wanderers'!$E$16</f>
         <v/>
       </c>
       <c r="E14" s="9">
-        <f>'Peterborough United'!$E$18</f>
+        <f>'Wycombe Wanderers'!$E$18</f>
         <v/>
       </c>
       <c r="F14" s="9">
-        <f>'Peterborough United'!$E$20</f>
+        <f>'Wycombe Wanderers'!$E$20</f>
         <v/>
       </c>
       <c r="G14" s="9">
-        <f>'Peterborough United'!$E$22</f>
+        <f>'Wycombe Wanderers'!$E$22</f>
         <v/>
       </c>
       <c r="H14" s="9">
-        <f>'Peterborough United'!$E$26</f>
+        <f>'Wycombe Wanderers'!$E$26</f>
         <v/>
       </c>
       <c r="I14" s="9">
-        <f>'Peterborough United'!$E$27</f>
+        <f>'Wycombe Wanderers'!$E$27</f>
         <v/>
       </c>
       <c r="J14" s="9">
-        <f>'Peterborough United'!$E$30</f>
+        <f>'Wycombe Wanderers'!$E$30</f>
         <v/>
       </c>
       <c r="K14" s="9">
-        <f>'Peterborough United'!$E$31</f>
+        <f>'Wycombe Wanderers'!$E$31</f>
         <v/>
       </c>
       <c r="L14" s="9">
-        <f>'Peterborough United'!$E$32</f>
+        <f>'Wycombe Wanderers'!$E$32</f>
         <v/>
       </c>
     </row>
@@ -27470,7 +27176,7 @@
         <v>0.25</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>-0.53</v>
+        <v>-0.54</v>
       </c>
       <c r="O6" s="9" t="n">
         <v>-0.3</v>
@@ -27558,7 +27264,7 @@
         <v>0.29</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="Q7" s="10" t="n">
         <v>0.35</v>
@@ -28419,7 +28125,7 @@
         <v>-0.04</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>-0.33</v>
+        <v>-0.34</v>
       </c>
       <c r="P3" s="10" t="n">
         <v>0.23</v>
@@ -28507,7 +28213,7 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -28662,16 +28368,16 @@
         <v>-0.09</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>0.54</v>
+        <v>0.51</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>-0.95</v>
+        <v>-0.99</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>-0.13</v>
+        <v>-0.14</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -28750,10 +28456,10 @@
         <v>-0.8100000000000001</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.03</v>
+        <v>-0.04</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>-0.24</v>
+        <v>-0.25</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -28808,34 +28514,34 @@
         <v>1.48</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>1.27</v>
+        <v>1.51</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>1.1</v>
+        <v>1.51</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>-0.33</v>
+        <v>-0.09</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>-0.38</v>
+        <v>0.03</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>-0.01</v>
+        <v>0.03</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>-0.26</v>
+        <v>-0.19</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.17</v>
       </c>
       <c r="O8" s="9" t="n">
-        <v>-0.65</v>
+        <v>-0.24</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>-0.13</v>
+        <v>-0.09</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.45</v>
+        <v>-0.39</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -28846,16 +28552,16 @@
         <v/>
       </c>
       <c r="T8" s="9" t="n">
-        <v>1.49</v>
+        <v>1.38</v>
       </c>
       <c r="U8" s="9" t="n">
         <v>1.46</v>
       </c>
       <c r="V8" s="9" t="n">
-        <v>0.03</v>
+        <v>-0.08</v>
       </c>
       <c r="W8" s="9" t="n">
-        <v>9.300000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="X8" s="9" t="n">
         <v>8.17</v>
@@ -29175,16 +28881,16 @@
         <v>5</v>
       </c>
       <c r="E36" s="19" t="n">
-        <v>0.39</v>
+        <v>0.35</v>
       </c>
       <c r="F36" s="19" t="n">
         <v>0.28</v>
       </c>
       <c r="G36" s="19" t="n">
-        <v>-0.5</v>
+        <v>-0.34</v>
       </c>
       <c r="H36" s="19" t="n">
-        <v>-0.54</v>
+        <v>-0.22</v>
       </c>
     </row>
     <row r="37">
@@ -29231,16 +28937,16 @@
         <v>12</v>
       </c>
       <c r="E38" s="21" t="n">
-        <v>0.21</v>
+        <v>0.19</v>
       </c>
       <c r="F38" s="21" t="n">
         <v>0.25</v>
       </c>
       <c r="G38" s="21" t="n">
-        <v>-0.18</v>
+        <v>-0.09</v>
       </c>
       <c r="H38" s="21" t="n">
-        <v>-0.38</v>
+        <v>-0.06</v>
       </c>
     </row>
   </sheetData>
@@ -29608,16 +29314,16 @@
         <v>0.54</v>
       </c>
       <c r="N2" s="9" t="n">
-        <v>-0.78</v>
+        <v>-0.82</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>0.23</v>
+        <v>0.2</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>-0.78</v>
+        <v>-0.82</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>0.23</v>
+        <v>0.2</v>
       </c>
       <c r="R2" s="9">
         <f>(H2-I2)-(F2-G2)</f>
@@ -29696,10 +29402,10 @@
         <v>0.5</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>-0.75</v>
+        <v>-0.77</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>0.36</v>
+        <v>0.35</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -29778,10 +29484,10 @@
         <v>0.01</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.52</v>
+        <v>-0.54</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -29860,10 +29566,10 @@
         <v>0.02</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>-0.48</v>
+        <v>-0.49</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -29936,16 +29642,16 @@
         <v>0.3</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>1.43</v>
+        <v>1.39</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>1.14</v>
+        <v>1.08</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.1</v>
+        <v>-0.11</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.38</v>
+        <v>0.36</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -30024,10 +29730,10 @@
         <v>-0.48</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.31</v>
+        <v>-0.32</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.24</v>
+        <v>0.22</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -30106,10 +29812,10 @@
         <v>-1.19</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>-0.11</v>
+        <v>-0.12</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0</v>
+        <v>-0.01</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -31049,7 +30755,7 @@
         <v>1.94</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="P4" s="9" t="n">
         <v>0.91</v>
@@ -31274,31 +30980,31 @@
         <v>1.05</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>2.62</v>
+        <v>2.44</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>0.59</v>
+        <v>0.58</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>0.91</v>
+        <v>0.73</v>
       </c>
       <c r="K7" s="10" t="n">
-        <v>-0.46</v>
+        <v>-0.47</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>0.93</v>
+        <v>0.9</v>
       </c>
       <c r="M7" s="10" t="n">
         <v>-0.35</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>1.46</v>
+        <v>1.28</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>-0.64</v>
+        <v>-0.65</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="Q7" s="10" t="n">
         <v>-0.36</v>
@@ -31312,16 +31018,16 @@
         <v/>
       </c>
       <c r="T7" s="10" t="n">
-        <v>2.55</v>
+        <v>2.5</v>
       </c>
       <c r="U7" s="10" t="n">
         <v>1.83</v>
       </c>
       <c r="V7" s="10" t="n">
-        <v>0.73</v>
+        <v>0.67</v>
       </c>
       <c r="W7" s="10" t="n">
-        <v>13.22</v>
+        <v>13.17</v>
       </c>
       <c r="X7" s="10" t="n">
         <v>9.050000000000001</v>
@@ -31641,13 +31347,13 @@
         <v>5</v>
       </c>
       <c r="E35" s="19" t="n">
-        <v>1.42</v>
+        <v>1.38</v>
       </c>
       <c r="F35" s="19" t="n">
-        <v>1.44</v>
+        <v>1.35</v>
       </c>
       <c r="G35" s="19" t="n">
-        <v>1.02</v>
+        <v>0.97</v>
       </c>
       <c r="H35" s="19" t="n">
         <v>0.9</v>
@@ -31697,16 +31403,16 @@
         <v>7</v>
       </c>
       <c r="E37" s="21" t="n">
-        <v>1.28</v>
+        <v>1.25</v>
       </c>
       <c r="F37" s="21" t="n">
-        <v>1.23</v>
+        <v>1.14</v>
       </c>
       <c r="G37" s="21" t="n">
-        <v>0.58</v>
+        <v>0.55</v>
       </c>
       <c r="H37" s="21" t="n">
-        <v>0.49</v>
+        <v>0.43</v>
       </c>
     </row>
   </sheetData>
@@ -32402,16 +32108,16 @@
         <v>0.08</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>-0.21</v>
+        <v>-0.27</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>0.64</v>
+        <v>0.6</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>1.06</v>
+        <v>1.04</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -32490,7 +32196,7 @@
         <v>0.2</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.6</v>
+        <v>0.59</v>
       </c>
       <c r="Q7" s="10" t="n">
         <v>0.28</v>
@@ -32548,34 +32254,34 @@
         <v>1.64</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>0.93</v>
+        <v>1.18</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>1.41</v>
+        <v>1.58</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>-0.43</v>
+        <v>-0.18</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>-0.23</v>
+        <v>-0.06</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>0.28</v>
+        <v>0.32</v>
       </c>
       <c r="M8" s="9" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="N8" s="9" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="O8" s="9" t="n">
+        <v>-0.49</v>
+      </c>
+      <c r="P8" s="9" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="Q8" s="9" t="n">
         <v>0.1</v>
-      </c>
-      <c r="N8" s="9" t="n">
-        <v>-0.44</v>
-      </c>
-      <c r="O8" s="9" t="n">
-        <v>-0.66</v>
-      </c>
-      <c r="P8" s="9" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="Q8" s="9" t="n">
-        <v>0.08</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -32586,16 +32292,16 @@
         <v/>
       </c>
       <c r="T8" s="9" t="n">
-        <v>1.01</v>
+        <v>1.1</v>
       </c>
       <c r="U8" s="9" t="n">
         <v>1.2</v>
       </c>
       <c r="V8" s="9" t="n">
-        <v>-0.18</v>
+        <v>-0.09</v>
       </c>
       <c r="W8" s="9" t="n">
-        <v>11.72</v>
+        <v>11.81</v>
       </c>
       <c r="X8" s="9" t="n">
         <v>10.97</v>
@@ -32915,16 +32621,16 @@
         <v>3</v>
       </c>
       <c r="E36" s="19" t="n">
-        <v>0.21</v>
+        <v>0.23</v>
       </c>
       <c r="F36" s="19" t="n">
-        <v>0.31</v>
+        <v>0.35</v>
       </c>
       <c r="G36" s="19" t="n">
-        <v>0.3</v>
+        <v>0.41</v>
       </c>
       <c r="H36" s="19" t="n">
-        <v>-0.59</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="37">
@@ -32971,13 +32677,13 @@
         <v>6</v>
       </c>
       <c r="E38" s="21" t="n">
-        <v>0.34</v>
+        <v>0.35</v>
       </c>
       <c r="F38" s="21" t="n">
         <v>0.8100000000000001</v>
       </c>
       <c r="G38" s="21" t="n">
-        <v>0.54</v>
+        <v>0.6</v>
       </c>
       <c r="H38" s="21" t="n">
         <v>0.19</v>
@@ -33436,7 +33142,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>-0.54</v>
+        <v>-0.55</v>
       </c>
       <c r="Q3" s="10" t="n">
         <v>0.02</v>
@@ -33512,16 +33218,16 @@
         <v>-0.16</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>-0.63</v>
+        <v>-0.67</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>-0.6</v>
+        <v>-0.67</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.57</v>
+        <v>-0.59</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.18</v>
+        <v>-0.21</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -33594,16 +33300,16 @@
         <v>-0.23</v>
       </c>
       <c r="N5" s="10" t="n">
+        <v>-0.63</v>
+      </c>
+      <c r="O5" s="10" t="n">
         <v>-0.5600000000000001</v>
       </c>
-      <c r="O5" s="10" t="n">
-        <v>-0.52</v>
-      </c>
       <c r="P5" s="10" t="n">
-        <v>-0.57</v>
+        <v>-0.6</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>-0.27</v>
+        <v>-0.29</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -33682,10 +33388,10 @@
         <v>0.28</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.27</v>
+        <v>-0.29</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>-0.16</v>
+        <v>-0.18</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -33764,10 +33470,10 @@
         <v>-0.38</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.16</v>
+        <v>-0.18</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>-0.2</v>
+        <v>-0.21</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -33846,10 +33552,10 @@
         <v>-0.77</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>-0.04</v>
+        <v>-0.06</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.32</v>
+        <v>-0.34</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -35096,34 +34802,34 @@
         <v>1.36</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>1.41</v>
+        <v>1.58</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>0.93</v>
+        <v>1.18</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>-0.23</v>
+        <v>-0.06</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>-0.43</v>
+        <v>-0.18</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>0.31</v>
+        <v>0.34</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>-0.38</v>
+        <v>-0.21</v>
       </c>
       <c r="O8" s="9" t="n">
-        <v>-1.01</v>
+        <v>-0.76</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.1</v>
+        <v>0.13</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.04</v>
+        <v>0</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -35134,16 +34840,16 @@
         <v/>
       </c>
       <c r="T8" s="9" t="n">
-        <v>1.71</v>
+        <v>1.65</v>
       </c>
       <c r="U8" s="9" t="n">
         <v>1.56</v>
       </c>
       <c r="V8" s="9" t="n">
-        <v>0.15</v>
+        <v>0.09</v>
       </c>
       <c r="W8" s="9" t="n">
-        <v>12.32</v>
+        <v>12.26</v>
       </c>
       <c r="X8" s="9" t="n">
         <v>11.01</v>
@@ -35491,16 +35197,16 @@
         <v>3</v>
       </c>
       <c r="E37" s="19" t="n">
-        <v>0.6</v>
+        <v>0.58</v>
       </c>
       <c r="F37" s="19" t="n">
-        <v>0.73</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G37" s="19" t="n">
-        <v>-0.24</v>
+        <v>-0.13</v>
       </c>
       <c r="H37" s="19" t="n">
-        <v>-0.43</v>
+        <v>-0.21</v>
       </c>
     </row>
     <row r="38">
@@ -35519,13 +35225,13 @@
         <v>10</v>
       </c>
       <c r="E38" s="21" t="n">
-        <v>0.39</v>
+        <v>0.38</v>
       </c>
       <c r="F38" s="21" t="n">
         <v>0.44</v>
       </c>
       <c r="G38" s="21" t="n">
-        <v>0.28</v>
+        <v>0.34</v>
       </c>
       <c r="H38" s="21" t="n">
         <v>-0.04</v>
@@ -36224,16 +35930,16 @@
         <v>0.59</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>-0.32</v>
+        <v>-0.36</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>0.74</v>
+        <v>0.71</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.59</v>
+        <v>0.58</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -36306,16 +36012,16 @@
         <v>0.3</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>0.54</v>
+        <v>0.51</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>-1.9</v>
+        <v>-1.94</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>0.58</v>
+        <v>0.57</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -36394,10 +36100,10 @@
         <v>-0.01</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -37334,16 +37040,16 @@
         <v>-0.01</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.52</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>-0.9399999999999999</v>
+        <v>-0.97</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.01</v>
+        <v>-0.02</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.19</v>
+        <v>-0.2</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -37416,16 +37122,16 @@
         <v>0.24</v>
       </c>
       <c r="N5" s="10" t="n">
-        <v>-0.31</v>
+        <v>-0.34</v>
       </c>
       <c r="O5" s="10" t="n">
-        <v>0.66</v>
+        <v>0.62</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>-0.08</v>
+        <v>-0.1</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -37504,10 +37210,10 @@
         <v>0.77</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.19</v>
+        <v>-0.2</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -37586,10 +37292,10 @@
         <v>-0.26</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>-0.26</v>
+        <v>-0.27</v>
       </c>
       <c r="Q7" s="10" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="R7" s="10">
         <f>(H7-I7)-(F7-G7)</f>
@@ -37668,10 +37374,10 @@
         <v>-1.62</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>-0.13</v>
+        <v>-0.14</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.33</v>
+        <v>-0.34</v>
       </c>
       <c r="R8" s="9">
         <f>(H8-I8)-(F8-G8)</f>
@@ -45751,28 +45457,28 @@
         <v>1.48</v>
       </c>
       <c r="H79" s="10" t="n">
-        <v>1.27</v>
+        <v>1.51</v>
       </c>
       <c r="I79" s="10" t="n">
-        <v>1.1</v>
+        <v>1.51</v>
       </c>
       <c r="J79" s="10" t="n">
-        <v>-0.33</v>
+        <v>-0.09</v>
       </c>
       <c r="K79" s="10" t="n">
-        <v>-0.38</v>
+        <v>0.03</v>
       </c>
       <c r="L79" s="10" t="n">
-        <v>0.06</v>
+        <v>-0.11</v>
       </c>
       <c r="M79" s="10" t="n">
-        <v>-0.71</v>
+        <v>-0.06</v>
       </c>
       <c r="N79" s="10" t="n">
-        <v>1.49</v>
+        <v>1.38</v>
       </c>
       <c r="O79" s="10" t="n">
-        <v>1.24</v>
+        <v>1.38</v>
       </c>
       <c r="P79" s="10" t="n">
         <v>1.46</v>
@@ -46049,25 +45755,25 @@
         <v>0.85</v>
       </c>
       <c r="I84" s="9" t="n">
-        <v>1.82</v>
+        <v>1.87</v>
       </c>
       <c r="J84" s="9" t="n">
         <v>-0.51</v>
       </c>
       <c r="K84" s="9" t="n">
-        <v>0.48</v>
+        <v>0.53</v>
       </c>
       <c r="L84" s="9" t="n">
-        <v>-0.99</v>
+        <v>-1.04</v>
       </c>
       <c r="M84" s="9" t="n">
-        <v>-0.03</v>
+        <v>0.02</v>
       </c>
       <c r="N84" s="9" t="n">
-        <v>0.74</v>
+        <v>0.72</v>
       </c>
       <c r="O84" s="9" t="n">
-        <v>2.04</v>
+        <v>2.06</v>
       </c>
       <c r="P84" s="9" t="n">
         <v>1.39</v>
@@ -46164,28 +45870,28 @@
         <v>1.64</v>
       </c>
       <c r="H86" s="9" t="n">
-        <v>0.93</v>
+        <v>1.18</v>
       </c>
       <c r="I86" s="9" t="n">
-        <v>1.41</v>
+        <v>1.58</v>
       </c>
       <c r="J86" s="9" t="n">
-        <v>-0.43</v>
+        <v>-0.18</v>
       </c>
       <c r="K86" s="9" t="n">
-        <v>-0.23</v>
+        <v>-0.06</v>
       </c>
       <c r="L86" s="9" t="n">
-        <v>-0.2</v>
+        <v>-0.12</v>
       </c>
       <c r="M86" s="9" t="n">
-        <v>-0.66</v>
+        <v>-0.24</v>
       </c>
       <c r="N86" s="9" t="n">
-        <v>1.01</v>
+        <v>1.1</v>
       </c>
       <c r="O86" s="9" t="n">
-        <v>1.71</v>
+        <v>1.65</v>
       </c>
       <c r="P86" s="9" t="n">
         <v>1.2</v>
@@ -46223,28 +45929,28 @@
         <v>1.05</v>
       </c>
       <c r="H87" s="10" t="n">
-        <v>2.62</v>
+        <v>2.44</v>
       </c>
       <c r="I87" s="10" t="n">
-        <v>0.59</v>
+        <v>0.58</v>
       </c>
       <c r="J87" s="10" t="n">
-        <v>0.91</v>
+        <v>0.73</v>
       </c>
       <c r="K87" s="10" t="n">
-        <v>-0.46</v>
+        <v>-0.47</v>
       </c>
       <c r="L87" s="10" t="n">
-        <v>1.37</v>
+        <v>1.2</v>
       </c>
       <c r="M87" s="10" t="n">
-        <v>0.45</v>
+        <v>0.26</v>
       </c>
       <c r="N87" s="10" t="n">
-        <v>2.55</v>
+        <v>2.5</v>
       </c>
       <c r="O87" s="10" t="n">
-        <v>0.32</v>
+        <v>0.35</v>
       </c>
       <c r="P87" s="10" t="n">
         <v>1.83</v>
@@ -46376,16 +46082,16 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>1.28</v>
+        <v>1.25</v>
       </c>
       <c r="C3" s="9" t="n">
-        <v>1.23</v>
+        <v>1.14</v>
       </c>
       <c r="D3" s="9" t="n">
-        <v>1.42</v>
+        <v>1.38</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>1.44</v>
+        <v>1.35</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>1.01</v>
@@ -46401,7 +46107,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>0.44</v>
+        <v>0.47</v>
       </c>
       <c r="C4" s="10" t="n">
         <v>0.2</v>
@@ -46413,10 +46119,10 @@
         <v>0.2</v>
       </c>
       <c r="F4" s="10" t="n">
-        <v>0.5</v>
+        <v>0.54</v>
       </c>
       <c r="G4" s="10" t="n">
-        <v>0.23</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="5">
@@ -46426,7 +46132,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.43</v>
+        <v>0.46</v>
       </c>
       <c r="C5" s="9" t="n">
         <v>0.18</v>
@@ -46438,7 +46144,7 @@
         <v>1.68</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>-0.19</v>
+        <v>-0.14</v>
       </c>
       <c r="G5" s="9" t="n">
         <v>-0.08</v>
@@ -46451,7 +46157,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>0.39</v>
+        <v>0.38</v>
       </c>
       <c r="C6" s="10" t="n">
         <v>0.44</v>
@@ -46463,10 +46169,10 @@
         <v>0.44</v>
       </c>
       <c r="F6" s="10" t="n">
-        <v>0.6</v>
+        <v>0.58</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>0.73</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -46476,16 +46182,16 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>0.34</v>
+        <v>0.35</v>
       </c>
       <c r="C7" s="9" t="n">
         <v>0.8100000000000001</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>0.21</v>
+        <v>0.23</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>0.31</v>
+        <v>0.35</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>0.5</v>
@@ -46522,51 +46228,51 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Peterborough United</t>
+          <t>Stevenage</t>
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.25</v>
+        <v>-0.18</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.39</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>0.28</v>
+        <v>-0.4</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>-0.02</v>
+        <v>0.4</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>-0.01</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Stevenage</t>
+          <t>Peterborough United</t>
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="C10" s="10" t="n">
-        <v>-0.18</v>
+        <v>0.25</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.35</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>-0.4</v>
+        <v>0.28</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>0.4</v>
+        <v>-0.02</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>0.19</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="11">
@@ -46701,7 +46407,7 @@
         </is>
       </c>
       <c r="B16" s="10" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.06</v>
       </c>
       <c r="C16" s="10" t="n">
         <v>-0.03</v>
@@ -46713,7 +46419,7 @@
         <v>0.01</v>
       </c>
       <c r="F16" s="10" t="n">
-        <v>-0.22</v>
+        <v>-0.21</v>
       </c>
       <c r="G16" s="10" t="n">
         <v>-0.19</v>
@@ -46857,7 +46563,7 @@
         <v>-0.08</v>
       </c>
       <c r="D22" s="10" t="n">
-        <v>-0.19</v>
+        <v>-0.2</v>
       </c>
       <c r="E22" s="10" t="n">
         <v>-0.39</v>
@@ -47166,51 +46872,51 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Peterborough United</t>
+          <t>Stevenage</t>
         </is>
       </c>
       <c r="B36" s="6" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C36" s="6" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D36" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E36" s="6" t="n">
         <v>5</v>
       </c>
       <c r="F36" s="6" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G36" s="6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>Stevenage</t>
+          <t>Peterborough United</t>
         </is>
       </c>
       <c r="B37" s="8" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C37" s="8" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D37" s="8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E37" s="8" t="n">
         <v>5</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G37" s="8" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="38">
@@ -48007,39 +47713,39 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Peterborough United</t>
+          <t>Stevenage</t>
         </is>
       </c>
       <c r="B8" s="13">
-        <f>'Peterborough United'!$E$22</f>
+        <f>'Stevenage'!$E$22</f>
         <v/>
       </c>
       <c r="C8" s="9">
-        <f>'Peterborough United'!$R$2</f>
+        <f>'Stevenage'!$R$2</f>
         <v/>
       </c>
       <c r="D8" s="9">
-        <f>'Peterborough United'!$R$3</f>
+        <f>'Stevenage'!$R$3</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>'Peterborough United'!$R$4</f>
+        <f>'Stevenage'!$R$4</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>'Peterborough United'!$R$5</f>
+        <f>'Stevenage'!$R$5</f>
         <v/>
       </c>
       <c r="G8" s="9">
-        <f>'Peterborough United'!$R$6</f>
+        <f>'Stevenage'!$R$6</f>
         <v/>
       </c>
       <c r="H8" s="9">
-        <f>'Peterborough United'!$R$7</f>
+        <f>'Stevenage'!$R$7</f>
         <v/>
       </c>
       <c r="I8" s="9">
-        <f>'Peterborough United'!$R$8</f>
+        <f>'Stevenage'!$R$8</f>
         <v/>
       </c>
       <c r="J8" s="6" t="n"/>
@@ -48047,39 +47753,39 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Stevenage</t>
+          <t>Peterborough United</t>
         </is>
       </c>
       <c r="B9" s="13">
-        <f>'Stevenage'!$E$22</f>
+        <f>'Peterborough United'!$E$22</f>
         <v/>
       </c>
       <c r="C9" s="9">
-        <f>'Stevenage'!$R$2</f>
+        <f>'Peterborough United'!$R$2</f>
         <v/>
       </c>
       <c r="D9" s="9">
-        <f>'Stevenage'!$R$3</f>
+        <f>'Peterborough United'!$R$3</f>
         <v/>
       </c>
       <c r="E9" s="9">
-        <f>'Stevenage'!$R$4</f>
+        <f>'Peterborough United'!$R$4</f>
         <v/>
       </c>
       <c r="F9" s="9">
-        <f>'Stevenage'!$R$5</f>
+        <f>'Peterborough United'!$R$5</f>
         <v/>
       </c>
       <c r="G9" s="9">
-        <f>'Stevenage'!$R$6</f>
+        <f>'Peterborough United'!$R$6</f>
         <v/>
       </c>
       <c r="H9" s="9">
-        <f>'Stevenage'!$R$7</f>
+        <f>'Peterborough United'!$R$7</f>
         <v/>
       </c>
       <c r="I9" s="9">
-        <f>'Stevenage'!$R$8</f>
+        <f>'Peterborough United'!$R$8</f>
         <v/>
       </c>
       <c r="J9" s="6" t="n"/>

</xml_diff>